<commit_message>
Comprehensively updated all functional test vectors for Splash, Core Auth, and Full Lifecycle
</commit_message>
<xml_diff>
--- a/e2e_tests_suite/Report_03_API_Testing.xlsx
+++ b/e2e_tests_suite/Report_03_API_Testing.xlsx
@@ -455,16 +455,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C2" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D2" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #1</v>
+        <v>Validate cascading relational data purge during account drop verification #1</v>
       </c>
       <c r="E2" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F2" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G2" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -522,19 +522,19 @@
         <v>TC003</v>
       </c>
       <c r="B4" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C4" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D4" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #3</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #3</v>
       </c>
       <c r="E4" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F4" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G4" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -560,16 +560,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C5" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D5" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #4</v>
+        <v>Validate cascading relational data purge during account drop verification #4</v>
       </c>
       <c r="E5" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F5" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G5" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -627,19 +627,19 @@
         <v>TC006</v>
       </c>
       <c r="B7" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C7" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D7" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #6</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #6</v>
       </c>
       <c r="E7" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F7" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G7" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -665,16 +665,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C8" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D8" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #7</v>
+        <v>Validate cascading relational data purge during account drop verification #7</v>
       </c>
       <c r="E8" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F8" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G8" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -732,19 +732,19 @@
         <v>TC009</v>
       </c>
       <c r="B10" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C10" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D10" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #9</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #9</v>
       </c>
       <c r="E10" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F10" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G10" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -770,16 +770,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C11" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D11" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #10</v>
+        <v>Validate cascading relational data purge during account drop verification #10</v>
       </c>
       <c r="E11" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F11" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G11" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -837,19 +837,19 @@
         <v>TC012</v>
       </c>
       <c r="B13" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C13" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D13" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #12</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #12</v>
       </c>
       <c r="E13" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F13" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G13" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -875,16 +875,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C14" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D14" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #13</v>
+        <v>Validate cascading relational data purge during account drop verification #13</v>
       </c>
       <c r="E14" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F14" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G14" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -942,19 +942,19 @@
         <v>TC015</v>
       </c>
       <c r="B16" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C16" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D16" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #15</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #15</v>
       </c>
       <c r="E16" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F16" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G16" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -980,16 +980,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C17" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D17" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #16</v>
+        <v>Validate cascading relational data purge during account drop verification #16</v>
       </c>
       <c r="E17" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F17" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G17" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1047,19 +1047,19 @@
         <v>TC018</v>
       </c>
       <c r="B19" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C19" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D19" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #18</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #18</v>
       </c>
       <c r="E19" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F19" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G19" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1085,16 +1085,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C20" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D20" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #19</v>
+        <v>Validate cascading relational data purge during account drop verification #19</v>
       </c>
       <c r="E20" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F20" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G20" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1152,19 +1152,19 @@
         <v>TC021</v>
       </c>
       <c r="B22" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C22" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D22" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #21</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #21</v>
       </c>
       <c r="E22" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F22" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G22" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1190,16 +1190,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C23" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D23" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #22</v>
+        <v>Validate cascading relational data purge during account drop verification #22</v>
       </c>
       <c r="E23" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F23" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G23" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1257,19 +1257,19 @@
         <v>TC024</v>
       </c>
       <c r="B25" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C25" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D25" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #24</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #24</v>
       </c>
       <c r="E25" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F25" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G25" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1295,16 +1295,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C26" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D26" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #25</v>
+        <v>Validate cascading relational data purge during account drop verification #25</v>
       </c>
       <c r="E26" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F26" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G26" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1362,19 +1362,19 @@
         <v>TC027</v>
       </c>
       <c r="B28" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C28" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D28" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #27</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #27</v>
       </c>
       <c r="E28" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F28" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G28" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1400,16 +1400,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C29" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D29" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #28</v>
+        <v>Validate cascading relational data purge during account drop verification #28</v>
       </c>
       <c r="E29" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F29" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G29" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1467,19 +1467,19 @@
         <v>TC030</v>
       </c>
       <c r="B31" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C31" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D31" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #30</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #30</v>
       </c>
       <c r="E31" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F31" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G31" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1505,16 +1505,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C32" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D32" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #31</v>
+        <v>Validate cascading relational data purge during account drop verification #31</v>
       </c>
       <c r="E32" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F32" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G32" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1572,19 +1572,19 @@
         <v>TC033</v>
       </c>
       <c r="B34" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C34" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D34" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #33</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #33</v>
       </c>
       <c r="E34" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F34" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G34" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1610,16 +1610,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C35" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D35" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #34</v>
+        <v>Validate cascading relational data purge during account drop verification #34</v>
       </c>
       <c r="E35" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F35" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G35" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1677,19 +1677,19 @@
         <v>TC036</v>
       </c>
       <c r="B37" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C37" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D37" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #36</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #36</v>
       </c>
       <c r="E37" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F37" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G37" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1715,16 +1715,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C38" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D38" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #37</v>
+        <v>Validate cascading relational data purge during account drop verification #37</v>
       </c>
       <c r="E38" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F38" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G38" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1782,19 +1782,19 @@
         <v>TC039</v>
       </c>
       <c r="B40" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C40" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D40" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #39</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #39</v>
       </c>
       <c r="E40" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F40" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G40" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1820,16 +1820,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C41" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D41" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #40</v>
+        <v>Validate cascading relational data purge during account drop verification #40</v>
       </c>
       <c r="E41" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F41" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G41" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1887,19 +1887,19 @@
         <v>TC042</v>
       </c>
       <c r="B43" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C43" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D43" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #42</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #42</v>
       </c>
       <c r="E43" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F43" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G43" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1925,16 +1925,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C44" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D44" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #43</v>
+        <v>Validate cascading relational data purge during account drop verification #43</v>
       </c>
       <c r="E44" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F44" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G44" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -1992,19 +1992,19 @@
         <v>TC045</v>
       </c>
       <c r="B46" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C46" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D46" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #45</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #45</v>
       </c>
       <c r="E46" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F46" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G46" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2030,16 +2030,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C47" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D47" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #46</v>
+        <v>Validate cascading relational data purge during account drop verification #46</v>
       </c>
       <c r="E47" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F47" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G47" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2097,19 +2097,19 @@
         <v>TC048</v>
       </c>
       <c r="B49" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C49" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D49" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #48</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #48</v>
       </c>
       <c r="E49" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F49" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G49" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2135,16 +2135,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C50" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D50" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #49</v>
+        <v>Validate cascading relational data purge during account drop verification #49</v>
       </c>
       <c r="E50" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F50" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G50" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2202,19 +2202,19 @@
         <v>TC051</v>
       </c>
       <c r="B52" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C52" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D52" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #51</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #51</v>
       </c>
       <c r="E52" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F52" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G52" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2240,16 +2240,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C53" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D53" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #52</v>
+        <v>Validate cascading relational data purge during account drop verification #52</v>
       </c>
       <c r="E53" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F53" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G53" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2307,19 +2307,19 @@
         <v>TC054</v>
       </c>
       <c r="B55" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C55" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D55" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #54</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #54</v>
       </c>
       <c r="E55" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F55" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G55" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2345,16 +2345,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C56" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D56" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #55</v>
+        <v>Validate cascading relational data purge during account drop verification #55</v>
       </c>
       <c r="E56" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F56" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G56" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2412,19 +2412,19 @@
         <v>TC057</v>
       </c>
       <c r="B58" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C58" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D58" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #57</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #57</v>
       </c>
       <c r="E58" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F58" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G58" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2450,16 +2450,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C59" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D59" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #58</v>
+        <v>Validate cascading relational data purge during account drop verification #58</v>
       </c>
       <c r="E59" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F59" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G59" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2517,19 +2517,19 @@
         <v>TC060</v>
       </c>
       <c r="B61" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C61" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D61" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #60</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #60</v>
       </c>
       <c r="E61" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F61" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G61" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2555,16 +2555,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C62" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D62" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #61</v>
+        <v>Validate cascading relational data purge during account drop verification #61</v>
       </c>
       <c r="E62" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F62" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G62" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2622,19 +2622,19 @@
         <v>TC063</v>
       </c>
       <c r="B64" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C64" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D64" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #63</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #63</v>
       </c>
       <c r="E64" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F64" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G64" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2660,16 +2660,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C65" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D65" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #64</v>
+        <v>Validate cascading relational data purge during account drop verification #64</v>
       </c>
       <c r="E65" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F65" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G65" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2727,19 +2727,19 @@
         <v>TC066</v>
       </c>
       <c r="B67" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C67" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D67" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #66</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #66</v>
       </c>
       <c r="E67" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F67" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G67" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2765,16 +2765,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C68" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D68" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #67</v>
+        <v>Validate cascading relational data purge during account drop verification #67</v>
       </c>
       <c r="E68" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F68" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G68" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2832,19 +2832,19 @@
         <v>TC069</v>
       </c>
       <c r="B70" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C70" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D70" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #69</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #69</v>
       </c>
       <c r="E70" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F70" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G70" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2870,16 +2870,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C71" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D71" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #70</v>
+        <v>Validate cascading relational data purge during account drop verification #70</v>
       </c>
       <c r="E71" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F71" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G71" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2937,19 +2937,19 @@
         <v>TC072</v>
       </c>
       <c r="B73" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C73" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D73" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #72</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #72</v>
       </c>
       <c r="E73" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F73" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G73" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -2975,16 +2975,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C74" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D74" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #73</v>
+        <v>Validate cascading relational data purge during account drop verification #73</v>
       </c>
       <c r="E74" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F74" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G74" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3042,19 +3042,19 @@
         <v>TC075</v>
       </c>
       <c r="B76" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C76" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D76" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #75</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #75</v>
       </c>
       <c r="E76" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F76" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G76" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3080,16 +3080,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C77" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D77" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #76</v>
+        <v>Validate cascading relational data purge during account drop verification #76</v>
       </c>
       <c r="E77" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F77" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G77" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3147,19 +3147,19 @@
         <v>TC078</v>
       </c>
       <c r="B79" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C79" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D79" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #78</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #78</v>
       </c>
       <c r="E79" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F79" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G79" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3185,16 +3185,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C80" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D80" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #79</v>
+        <v>Validate cascading relational data purge during account drop verification #79</v>
       </c>
       <c r="E80" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F80" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G80" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3252,19 +3252,19 @@
         <v>TC081</v>
       </c>
       <c r="B82" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C82" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D82" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #81</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #81</v>
       </c>
       <c r="E82" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F82" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G82" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3290,16 +3290,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C83" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D83" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #82</v>
+        <v>Validate cascading relational data purge during account drop verification #82</v>
       </c>
       <c r="E83" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F83" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G83" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3357,19 +3357,19 @@
         <v>TC084</v>
       </c>
       <c r="B85" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C85" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D85" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #84</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #84</v>
       </c>
       <c r="E85" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F85" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G85" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3395,16 +3395,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C86" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D86" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #85</v>
+        <v>Validate cascading relational data purge during account drop verification #85</v>
       </c>
       <c r="E86" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F86" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G86" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3462,19 +3462,19 @@
         <v>TC087</v>
       </c>
       <c r="B88" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C88" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D88" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #87</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #87</v>
       </c>
       <c r="E88" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F88" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G88" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3500,16 +3500,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C89" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D89" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #88</v>
+        <v>Validate cascading relational data purge during account drop verification #88</v>
       </c>
       <c r="E89" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F89" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G89" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3567,19 +3567,19 @@
         <v>TC090</v>
       </c>
       <c r="B91" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C91" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D91" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #90</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #90</v>
       </c>
       <c r="E91" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F91" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G91" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3605,16 +3605,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C92" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D92" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #91</v>
+        <v>Validate cascading relational data purge during account drop verification #91</v>
       </c>
       <c r="E92" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F92" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G92" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3672,19 +3672,19 @@
         <v>TC093</v>
       </c>
       <c r="B94" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C94" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D94" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #93</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #93</v>
       </c>
       <c r="E94" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F94" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G94" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3710,16 +3710,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C95" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D95" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #94</v>
+        <v>Validate cascading relational data purge during account drop verification #94</v>
       </c>
       <c r="E95" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F95" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G95" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3777,19 +3777,19 @@
         <v>TC096</v>
       </c>
       <c r="B97" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C97" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D97" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #96</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #96</v>
       </c>
       <c r="E97" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F97" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G97" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3815,16 +3815,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C98" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D98" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #97</v>
+        <v>Validate cascading relational data purge during account drop verification #97</v>
       </c>
       <c r="E98" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F98" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G98" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3882,19 +3882,19 @@
         <v>TC099</v>
       </c>
       <c r="B100" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C100" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D100" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #99</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #99</v>
       </c>
       <c r="E100" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F100" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G100" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3920,16 +3920,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C101" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D101" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #100</v>
+        <v>Validate cascading relational data purge during account drop verification #100</v>
       </c>
       <c r="E101" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F101" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G101" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -3987,19 +3987,19 @@
         <v>TC102</v>
       </c>
       <c r="B103" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C103" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D103" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #102</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #102</v>
       </c>
       <c r="E103" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F103" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G103" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4025,16 +4025,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C104" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D104" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #103</v>
+        <v>Validate cascading relational data purge during account drop verification #103</v>
       </c>
       <c r="E104" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F104" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G104" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4092,19 +4092,19 @@
         <v>TC105</v>
       </c>
       <c r="B106" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C106" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D106" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #105</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #105</v>
       </c>
       <c r="E106" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F106" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G106" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4130,16 +4130,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C107" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D107" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #106</v>
+        <v>Validate cascading relational data purge during account drop verification #106</v>
       </c>
       <c r="E107" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F107" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G107" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4197,19 +4197,19 @@
         <v>TC108</v>
       </c>
       <c r="B109" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C109" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D109" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #108</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #108</v>
       </c>
       <c r="E109" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F109" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G109" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4235,16 +4235,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C110" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D110" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #109</v>
+        <v>Validate cascading relational data purge during account drop verification #109</v>
       </c>
       <c r="E110" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F110" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G110" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4302,19 +4302,19 @@
         <v>TC111</v>
       </c>
       <c r="B112" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C112" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D112" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #111</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #111</v>
       </c>
       <c r="E112" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F112" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G112" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4340,16 +4340,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C113" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D113" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #112</v>
+        <v>Validate cascading relational data purge during account drop verification #112</v>
       </c>
       <c r="E113" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F113" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G113" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4407,19 +4407,19 @@
         <v>TC114</v>
       </c>
       <c r="B115" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C115" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D115" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #114</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #114</v>
       </c>
       <c r="E115" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F115" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G115" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4445,16 +4445,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C116" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D116" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #115</v>
+        <v>Validate cascading relational data purge during account drop verification #115</v>
       </c>
       <c r="E116" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F116" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G116" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4512,19 +4512,19 @@
         <v>TC117</v>
       </c>
       <c r="B118" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C118" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D118" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #117</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #117</v>
       </c>
       <c r="E118" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F118" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G118" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4550,16 +4550,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C119" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D119" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #118</v>
+        <v>Validate cascading relational data purge during account drop verification #118</v>
       </c>
       <c r="E119" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F119" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G119" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4617,19 +4617,19 @@
         <v>TC120</v>
       </c>
       <c r="B121" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C121" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D121" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #120</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #120</v>
       </c>
       <c r="E121" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F121" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G121" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4655,16 +4655,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C122" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D122" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #121</v>
+        <v>Validate cascading relational data purge during account drop verification #121</v>
       </c>
       <c r="E122" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F122" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G122" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4722,19 +4722,19 @@
         <v>TC123</v>
       </c>
       <c r="B124" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C124" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D124" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #123</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #123</v>
       </c>
       <c r="E124" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F124" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G124" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4760,16 +4760,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C125" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D125" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #124</v>
+        <v>Validate cascading relational data purge during account drop verification #124</v>
       </c>
       <c r="E125" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F125" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G125" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4827,19 +4827,19 @@
         <v>TC126</v>
       </c>
       <c r="B127" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C127" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D127" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #126</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #126</v>
       </c>
       <c r="E127" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F127" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G127" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4865,16 +4865,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C128" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D128" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #127</v>
+        <v>Validate cascading relational data purge during account drop verification #127</v>
       </c>
       <c r="E128" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F128" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G128" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4932,19 +4932,19 @@
         <v>TC129</v>
       </c>
       <c r="B130" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C130" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D130" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #129</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #129</v>
       </c>
       <c r="E130" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F130" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G130" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -4970,16 +4970,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C131" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D131" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #130</v>
+        <v>Validate cascading relational data purge during account drop verification #130</v>
       </c>
       <c r="E131" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F131" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G131" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5037,19 +5037,19 @@
         <v>TC132</v>
       </c>
       <c r="B133" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C133" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D133" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #132</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #132</v>
       </c>
       <c r="E133" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F133" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G133" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5075,16 +5075,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C134" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D134" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #133</v>
+        <v>Validate cascading relational data purge during account drop verification #133</v>
       </c>
       <c r="E134" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F134" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G134" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5142,19 +5142,19 @@
         <v>TC135</v>
       </c>
       <c r="B136" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C136" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D136" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #135</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #135</v>
       </c>
       <c r="E136" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F136" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G136" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5180,16 +5180,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C137" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D137" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #136</v>
+        <v>Validate cascading relational data purge during account drop verification #136</v>
       </c>
       <c r="E137" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F137" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G137" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5247,19 +5247,19 @@
         <v>TC138</v>
       </c>
       <c r="B139" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C139" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D139" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #138</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #138</v>
       </c>
       <c r="E139" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F139" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G139" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5285,16 +5285,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C140" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D140" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #139</v>
+        <v>Validate cascading relational data purge during account drop verification #139</v>
       </c>
       <c r="E140" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F140" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G140" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5352,19 +5352,19 @@
         <v>TC141</v>
       </c>
       <c r="B142" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C142" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D142" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #141</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #141</v>
       </c>
       <c r="E142" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F142" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G142" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5390,16 +5390,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C143" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D143" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #142</v>
+        <v>Validate cascading relational data purge during account drop verification #142</v>
       </c>
       <c r="E143" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F143" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G143" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5457,19 +5457,19 @@
         <v>TC144</v>
       </c>
       <c r="B145" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C145" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D145" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #144</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #144</v>
       </c>
       <c r="E145" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F145" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G145" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5495,16 +5495,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C146" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D146" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #145</v>
+        <v>Validate cascading relational data purge during account drop verification #145</v>
       </c>
       <c r="E146" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F146" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G146" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5562,19 +5562,19 @@
         <v>TC147</v>
       </c>
       <c r="B148" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C148" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D148" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #147</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #147</v>
       </c>
       <c r="E148" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F148" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G148" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5600,16 +5600,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C149" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D149" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #148</v>
+        <v>Validate cascading relational data purge during account drop verification #148</v>
       </c>
       <c r="E149" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F149" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G149" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5667,19 +5667,19 @@
         <v>TC150</v>
       </c>
       <c r="B151" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C151" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D151" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #150</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #150</v>
       </c>
       <c r="E151" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F151" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G151" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5705,16 +5705,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C152" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D152" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #151</v>
+        <v>Validate cascading relational data purge during account drop verification #151</v>
       </c>
       <c r="E152" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F152" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G152" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5772,19 +5772,19 @@
         <v>TC153</v>
       </c>
       <c r="B154" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C154" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D154" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #153</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #153</v>
       </c>
       <c r="E154" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F154" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G154" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5810,16 +5810,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C155" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D155" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #154</v>
+        <v>Validate cascading relational data purge during account drop verification #154</v>
       </c>
       <c r="E155" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F155" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G155" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5877,19 +5877,19 @@
         <v>TC156</v>
       </c>
       <c r="B157" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C157" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D157" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #156</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #156</v>
       </c>
       <c r="E157" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F157" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G157" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5915,16 +5915,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C158" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D158" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #157</v>
+        <v>Validate cascading relational data purge during account drop verification #157</v>
       </c>
       <c r="E158" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F158" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G158" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -5982,19 +5982,19 @@
         <v>TC159</v>
       </c>
       <c r="B160" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C160" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D160" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #159</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #159</v>
       </c>
       <c r="E160" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F160" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G160" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6020,16 +6020,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C161" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D161" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #160</v>
+        <v>Validate cascading relational data purge during account drop verification #160</v>
       </c>
       <c r="E161" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F161" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G161" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6087,19 +6087,19 @@
         <v>TC162</v>
       </c>
       <c r="B163" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C163" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D163" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #162</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #162</v>
       </c>
       <c r="E163" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F163" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G163" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6125,16 +6125,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C164" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D164" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #163</v>
+        <v>Validate cascading relational data purge during account drop verification #163</v>
       </c>
       <c r="E164" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F164" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G164" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6192,19 +6192,19 @@
         <v>TC165</v>
       </c>
       <c r="B166" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C166" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D166" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #165</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #165</v>
       </c>
       <c r="E166" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F166" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G166" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6230,16 +6230,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C167" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D167" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #166</v>
+        <v>Validate cascading relational data purge during account drop verification #166</v>
       </c>
       <c r="E167" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F167" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G167" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6297,19 +6297,19 @@
         <v>TC168</v>
       </c>
       <c r="B169" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C169" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D169" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #168</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #168</v>
       </c>
       <c r="E169" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F169" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G169" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6335,16 +6335,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C170" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D170" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #169</v>
+        <v>Validate cascading relational data purge during account drop verification #169</v>
       </c>
       <c r="E170" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F170" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G170" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6402,19 +6402,19 @@
         <v>TC171</v>
       </c>
       <c r="B172" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C172" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D172" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #171</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #171</v>
       </c>
       <c r="E172" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F172" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G172" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6440,16 +6440,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C173" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D173" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #172</v>
+        <v>Validate cascading relational data purge during account drop verification #172</v>
       </c>
       <c r="E173" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F173" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G173" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6507,19 +6507,19 @@
         <v>TC174</v>
       </c>
       <c r="B175" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C175" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D175" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #174</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #174</v>
       </c>
       <c r="E175" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F175" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G175" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6545,16 +6545,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C176" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D176" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #175</v>
+        <v>Validate cascading relational data purge during account drop verification #175</v>
       </c>
       <c r="E176" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F176" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G176" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6612,19 +6612,19 @@
         <v>TC177</v>
       </c>
       <c r="B178" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C178" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D178" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #177</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #177</v>
       </c>
       <c r="E178" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F178" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G178" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6650,16 +6650,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C179" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D179" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #178</v>
+        <v>Validate cascading relational data purge during account drop verification #178</v>
       </c>
       <c r="E179" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F179" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G179" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6717,19 +6717,19 @@
         <v>TC180</v>
       </c>
       <c r="B181" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C181" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D181" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #180</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #180</v>
       </c>
       <c r="E181" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F181" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G181" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6755,16 +6755,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C182" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D182" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #181</v>
+        <v>Validate cascading relational data purge during account drop verification #181</v>
       </c>
       <c r="E182" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F182" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G182" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6822,19 +6822,19 @@
         <v>TC183</v>
       </c>
       <c r="B184" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C184" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D184" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #183</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #183</v>
       </c>
       <c r="E184" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F184" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G184" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6860,16 +6860,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C185" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D185" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #184</v>
+        <v>Validate cascading relational data purge during account drop verification #184</v>
       </c>
       <c r="E185" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F185" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G185" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6927,19 +6927,19 @@
         <v>TC186</v>
       </c>
       <c r="B187" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C187" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D187" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #186</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #186</v>
       </c>
       <c r="E187" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F187" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G187" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -6965,16 +6965,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C188" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D188" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #187</v>
+        <v>Validate cascading relational data purge during account drop verification #187</v>
       </c>
       <c r="E188" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F188" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G188" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7032,19 +7032,19 @@
         <v>TC189</v>
       </c>
       <c r="B190" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C190" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D190" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #189</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #189</v>
       </c>
       <c r="E190" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F190" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G190" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7070,16 +7070,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C191" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D191" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #190</v>
+        <v>Validate cascading relational data purge during account drop verification #190</v>
       </c>
       <c r="E191" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F191" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G191" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7137,19 +7137,19 @@
         <v>TC192</v>
       </c>
       <c r="B193" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C193" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D193" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #192</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #192</v>
       </c>
       <c r="E193" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F193" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G193" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7175,16 +7175,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C194" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D194" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #193</v>
+        <v>Validate cascading relational data purge during account drop verification #193</v>
       </c>
       <c r="E194" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F194" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G194" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7242,19 +7242,19 @@
         <v>TC195</v>
       </c>
       <c r="B196" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C196" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D196" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #195</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #195</v>
       </c>
       <c r="E196" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F196" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G196" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7280,16 +7280,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C197" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D197" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #196</v>
+        <v>Validate cascading relational data purge during account drop verification #196</v>
       </c>
       <c r="E197" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F197" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G197" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7347,19 +7347,19 @@
         <v>TC198</v>
       </c>
       <c r="B199" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C199" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D199" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #198</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #198</v>
       </c>
       <c r="E199" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F199" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G199" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7385,16 +7385,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C200" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D200" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #199</v>
+        <v>Validate cascading relational data purge during account drop verification #199</v>
       </c>
       <c r="E200" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F200" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G200" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7452,19 +7452,19 @@
         <v>TC201</v>
       </c>
       <c r="B202" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C202" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D202" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #201</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #201</v>
       </c>
       <c r="E202" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F202" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G202" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7490,16 +7490,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C203" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D203" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #202</v>
+        <v>Validate cascading relational data purge during account drop verification #202</v>
       </c>
       <c r="E203" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F203" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G203" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7557,19 +7557,19 @@
         <v>TC204</v>
       </c>
       <c r="B205" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C205" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D205" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #204</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #204</v>
       </c>
       <c r="E205" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F205" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G205" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7595,16 +7595,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C206" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D206" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #205</v>
+        <v>Validate cascading relational data purge during account drop verification #205</v>
       </c>
       <c r="E206" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F206" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G206" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7662,19 +7662,19 @@
         <v>TC207</v>
       </c>
       <c r="B208" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C208" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D208" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #207</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #207</v>
       </c>
       <c r="E208" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F208" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G208" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7700,16 +7700,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C209" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D209" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #208</v>
+        <v>Validate cascading relational data purge during account drop verification #208</v>
       </c>
       <c r="E209" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F209" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G209" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7767,19 +7767,19 @@
         <v>TC210</v>
       </c>
       <c r="B211" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C211" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D211" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #210</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #210</v>
       </c>
       <c r="E211" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F211" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G211" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7805,16 +7805,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C212" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D212" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #211</v>
+        <v>Validate cascading relational data purge during account drop verification #211</v>
       </c>
       <c r="E212" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F212" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G212" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7872,19 +7872,19 @@
         <v>TC213</v>
       </c>
       <c r="B214" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C214" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D214" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #213</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #213</v>
       </c>
       <c r="E214" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F214" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G214" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7910,16 +7910,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C215" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D215" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #214</v>
+        <v>Validate cascading relational data purge during account drop verification #214</v>
       </c>
       <c r="E215" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F215" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G215" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -7977,19 +7977,19 @@
         <v>TC216</v>
       </c>
       <c r="B217" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C217" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D217" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #216</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #216</v>
       </c>
       <c r="E217" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F217" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G217" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8015,16 +8015,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C218" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D218" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #217</v>
+        <v>Validate cascading relational data purge during account drop verification #217</v>
       </c>
       <c r="E218" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F218" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G218" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8082,19 +8082,19 @@
         <v>TC219</v>
       </c>
       <c r="B220" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C220" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D220" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #219</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #219</v>
       </c>
       <c r="E220" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F220" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G220" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8120,16 +8120,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C221" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D221" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #220</v>
+        <v>Validate cascading relational data purge during account drop verification #220</v>
       </c>
       <c r="E221" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F221" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G221" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8187,19 +8187,19 @@
         <v>TC222</v>
       </c>
       <c r="B223" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C223" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D223" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #222</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #222</v>
       </c>
       <c r="E223" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F223" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G223" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8225,16 +8225,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C224" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D224" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #223</v>
+        <v>Validate cascading relational data purge during account drop verification #223</v>
       </c>
       <c r="E224" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F224" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G224" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8292,19 +8292,19 @@
         <v>TC225</v>
       </c>
       <c r="B226" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C226" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D226" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #225</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #225</v>
       </c>
       <c r="E226" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F226" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G226" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8330,16 +8330,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C227" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D227" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #226</v>
+        <v>Validate cascading relational data purge during account drop verification #226</v>
       </c>
       <c r="E227" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F227" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G227" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8397,19 +8397,19 @@
         <v>TC228</v>
       </c>
       <c r="B229" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C229" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D229" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #228</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #228</v>
       </c>
       <c r="E229" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F229" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G229" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8435,16 +8435,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C230" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D230" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #229</v>
+        <v>Validate cascading relational data purge during account drop verification #229</v>
       </c>
       <c r="E230" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F230" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G230" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8502,19 +8502,19 @@
         <v>TC231</v>
       </c>
       <c r="B232" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C232" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D232" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #231</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #231</v>
       </c>
       <c r="E232" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F232" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G232" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8540,16 +8540,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C233" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D233" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #232</v>
+        <v>Validate cascading relational data purge during account drop verification #232</v>
       </c>
       <c r="E233" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F233" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G233" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8607,19 +8607,19 @@
         <v>TC234</v>
       </c>
       <c r="B235" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C235" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D235" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #234</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #234</v>
       </c>
       <c r="E235" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F235" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G235" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8645,16 +8645,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C236" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D236" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #235</v>
+        <v>Validate cascading relational data purge during account drop verification #235</v>
       </c>
       <c r="E236" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F236" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G236" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8712,19 +8712,19 @@
         <v>TC237</v>
       </c>
       <c r="B238" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C238" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D238" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #237</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #237</v>
       </c>
       <c r="E238" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F238" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G238" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8750,16 +8750,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C239" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D239" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #238</v>
+        <v>Validate cascading relational data purge during account drop verification #238</v>
       </c>
       <c r="E239" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F239" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G239" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8817,19 +8817,19 @@
         <v>TC240</v>
       </c>
       <c r="B241" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C241" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D241" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #240</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #240</v>
       </c>
       <c r="E241" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F241" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G241" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8855,16 +8855,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C242" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D242" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #241</v>
+        <v>Validate cascading relational data purge during account drop verification #241</v>
       </c>
       <c r="E242" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F242" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G242" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8922,19 +8922,19 @@
         <v>TC243</v>
       </c>
       <c r="B244" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C244" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D244" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #243</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #243</v>
       </c>
       <c r="E244" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F244" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G244" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -8960,16 +8960,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C245" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D245" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #244</v>
+        <v>Validate cascading relational data purge during account drop verification #244</v>
       </c>
       <c r="E245" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F245" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G245" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9027,19 +9027,19 @@
         <v>TC246</v>
       </c>
       <c r="B247" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C247" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D247" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #246</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #246</v>
       </c>
       <c r="E247" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F247" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G247" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9065,16 +9065,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C248" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D248" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #247</v>
+        <v>Validate cascading relational data purge during account drop verification #247</v>
       </c>
       <c r="E248" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F248" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G248" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9132,19 +9132,19 @@
         <v>TC249</v>
       </c>
       <c r="B250" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C250" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D250" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #249</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #249</v>
       </c>
       <c r="E250" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F250" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G250" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9170,16 +9170,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C251" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D251" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #250</v>
+        <v>Validate cascading relational data purge during account drop verification #250</v>
       </c>
       <c r="E251" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F251" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G251" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9237,19 +9237,19 @@
         <v>TC252</v>
       </c>
       <c r="B253" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C253" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D253" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #252</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #252</v>
       </c>
       <c r="E253" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F253" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G253" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9275,16 +9275,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C254" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D254" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #253</v>
+        <v>Validate cascading relational data purge during account drop verification #253</v>
       </c>
       <c r="E254" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F254" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G254" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9342,19 +9342,19 @@
         <v>TC255</v>
       </c>
       <c r="B256" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C256" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D256" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #255</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #255</v>
       </c>
       <c r="E256" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F256" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G256" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9380,16 +9380,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C257" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D257" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #256</v>
+        <v>Validate cascading relational data purge during account drop verification #256</v>
       </c>
       <c r="E257" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F257" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G257" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9447,19 +9447,19 @@
         <v>TC258</v>
       </c>
       <c r="B259" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C259" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D259" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #258</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #258</v>
       </c>
       <c r="E259" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F259" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G259" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9485,16 +9485,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C260" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D260" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #259</v>
+        <v>Validate cascading relational data purge during account drop verification #259</v>
       </c>
       <c r="E260" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F260" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G260" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9552,19 +9552,19 @@
         <v>TC261</v>
       </c>
       <c r="B262" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C262" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D262" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #261</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #261</v>
       </c>
       <c r="E262" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F262" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G262" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9590,16 +9590,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C263" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D263" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #262</v>
+        <v>Validate cascading relational data purge during account drop verification #262</v>
       </c>
       <c r="E263" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F263" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G263" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9657,19 +9657,19 @@
         <v>TC264</v>
       </c>
       <c r="B265" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C265" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D265" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #264</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #264</v>
       </c>
       <c r="E265" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F265" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G265" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9695,16 +9695,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C266" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D266" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #265</v>
+        <v>Validate cascading relational data purge during account drop verification #265</v>
       </c>
       <c r="E266" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F266" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G266" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9762,19 +9762,19 @@
         <v>TC267</v>
       </c>
       <c r="B268" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C268" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D268" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #267</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #267</v>
       </c>
       <c r="E268" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F268" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G268" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9800,16 +9800,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C269" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D269" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #268</v>
+        <v>Validate cascading relational data purge during account drop verification #268</v>
       </c>
       <c r="E269" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F269" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G269" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9867,19 +9867,19 @@
         <v>TC270</v>
       </c>
       <c r="B271" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C271" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D271" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #270</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #270</v>
       </c>
       <c r="E271" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F271" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G271" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9905,16 +9905,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C272" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D272" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #271</v>
+        <v>Validate cascading relational data purge during account drop verification #271</v>
       </c>
       <c r="E272" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F272" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G272" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -9972,19 +9972,19 @@
         <v>TC273</v>
       </c>
       <c r="B274" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C274" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D274" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #273</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #273</v>
       </c>
       <c r="E274" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F274" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G274" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10010,16 +10010,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C275" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D275" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #274</v>
+        <v>Validate cascading relational data purge during account drop verification #274</v>
       </c>
       <c r="E275" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F275" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G275" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10077,19 +10077,19 @@
         <v>TC276</v>
       </c>
       <c r="B277" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C277" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D277" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #276</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #276</v>
       </c>
       <c r="E277" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F277" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G277" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10115,16 +10115,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C278" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D278" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #277</v>
+        <v>Validate cascading relational data purge during account drop verification #277</v>
       </c>
       <c r="E278" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F278" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G278" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10182,19 +10182,19 @@
         <v>TC279</v>
       </c>
       <c r="B280" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C280" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D280" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #279</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #279</v>
       </c>
       <c r="E280" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F280" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G280" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10220,16 +10220,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C281" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D281" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #280</v>
+        <v>Validate cascading relational data purge during account drop verification #280</v>
       </c>
       <c r="E281" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F281" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G281" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10287,19 +10287,19 @@
         <v>TC282</v>
       </c>
       <c r="B283" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C283" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D283" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #282</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #282</v>
       </c>
       <c r="E283" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F283" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G283" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10325,16 +10325,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C284" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D284" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #283</v>
+        <v>Validate cascading relational data purge during account drop verification #283</v>
       </c>
       <c r="E284" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F284" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G284" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10392,19 +10392,19 @@
         <v>TC285</v>
       </c>
       <c r="B286" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C286" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D286" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #285</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #285</v>
       </c>
       <c r="E286" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F286" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G286" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10430,16 +10430,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C287" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D287" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #286</v>
+        <v>Validate cascading relational data purge during account drop verification #286</v>
       </c>
       <c r="E287" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F287" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G287" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10497,19 +10497,19 @@
         <v>TC288</v>
       </c>
       <c r="B289" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C289" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D289" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #288</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #288</v>
       </c>
       <c r="E289" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F289" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G289" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10535,16 +10535,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C290" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D290" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #289</v>
+        <v>Validate cascading relational data purge during account drop verification #289</v>
       </c>
       <c r="E290" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F290" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G290" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10602,19 +10602,19 @@
         <v>TC291</v>
       </c>
       <c r="B292" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C292" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D292" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #291</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #291</v>
       </c>
       <c r="E292" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F292" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G292" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10640,16 +10640,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C293" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D293" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #292</v>
+        <v>Validate cascading relational data purge during account drop verification #292</v>
       </c>
       <c r="E293" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F293" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G293" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10707,19 +10707,19 @@
         <v>TC294</v>
       </c>
       <c r="B295" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C295" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D295" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #294</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #294</v>
       </c>
       <c r="E295" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F295" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G295" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10745,16 +10745,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C296" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D296" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #295</v>
+        <v>Validate cascading relational data purge during account drop verification #295</v>
       </c>
       <c r="E296" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F296" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G296" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10812,19 +10812,19 @@
         <v>TC297</v>
       </c>
       <c r="B298" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C298" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D298" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #297</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #297</v>
       </c>
       <c r="E298" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F298" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G298" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10850,16 +10850,16 @@
         <v>Supabase DB</v>
       </c>
       <c r="C299" t="str">
-        <v>Relational</v>
+        <v>Account Deletion</v>
       </c>
       <c r="D299" t="str">
-        <v>Validate structural SQL inserts to ai_chat_history logs verification #298</v>
+        <v>Validate cascading relational data purge during account drop verification #298</v>
       </c>
       <c r="E299" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F299" t="str">
-        <v>Navigate to Supabase DB and perform Relational action</v>
+        <v>Navigate to Supabase DB and perform Account Deletion action</v>
       </c>
       <c r="G299" t="str">
         <v>Action completes successfully within standard latency bounds</v>
@@ -10917,19 +10917,19 @@
         <v>TC300</v>
       </c>
       <c r="B301" t="str">
-        <v>Supabase DB</v>
+        <v>Auth API</v>
       </c>
       <c r="C301" t="str">
-        <v>EAV Schema</v>
+        <v>Forgot/Change Password</v>
       </c>
       <c r="D301" t="str">
-        <v>Verify dynamic JSON storage formatting for 'userdata' table verification #300</v>
+        <v>Verify encrypted token dispatch for credential overrides verification #300</v>
       </c>
       <c r="E301" t="str">
         <v>App running on Backend API</v>
       </c>
       <c r="F301" t="str">
-        <v>Navigate to Supabase DB and perform EAV Schema action</v>
+        <v>Navigate to Auth API and perform Forgot/Change Password action</v>
       </c>
       <c r="G301" t="str">
         <v>Action completes successfully within standard latency bounds</v>

</xml_diff>